<commit_message>
chore(execucao): atualiza artefatos da coleta e auditoria
Adiciona os PDFs de respostas do questionario e a planilha de relacao das evidencias no Google Drive.

Atualiza artefatos da execucao da auditoria, questionario de comentarios do gestor e anexos relacionados.

Ajusta a redacao das recomendacoes para reforcar proporcionalidade ao porte, maturidade, complexidade e risco das organizacoes auditadas.
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados.xlsx
@@ -407,11 +407,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A3:D5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="4">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -1514,7 +1512,7 @@
       <c r="O14" s="6" t="n"/>
       <c r="P14" s="6" t="inlineStr">
         <is>
-          <t>institua formalmente Comitê de TIC ou instância equivalente, atentando-se, minimamente, em definir sua composição, competências, periodicidade de reuniões, forma de registro das deliberações e acompanhamento dos encaminhamentos</t>
+          <t>institua formalmente Comitê de TIC ou instância equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em definir sua composição, competências, periodicidade de reuniões, forma de registro das deliberações e acompanhamento dos encaminhamentos</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1568,7 @@
       <c r="O15" s="6" t="n"/>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, atentando-se, minimamente, em realizar reuniões periódicas, registrar atas, deliberações e encaminhamentos e acompanhar as decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em realizar reuniões periódicas, registrar deliberações e acompanhar decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1624,7 @@
       <c r="O16" s="6" t="n"/>
       <c r="P16" s="6" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, atentando-se, minimamente, em realizar reuniões periódicas, registrar atas, deliberações e encaminhamentos e acompanhar as decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em realizar reuniões periódicas, registrar deliberações e acompanhar decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1680,7 @@
       <c r="O17" s="6" t="n"/>
       <c r="P17" s="6" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1736,7 @@
       <c r="O18" s="6" t="n"/>
       <c r="P18" s="6" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1792,7 @@
       <c r="O19" s="6" t="n"/>
       <c r="P19" s="6" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1848,7 @@
       <c r="O20" s="6" t="n"/>
       <c r="P20" s="6" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3416,7 @@
       <c r="O48" s="6" t="n"/>
       <c r="P48" s="6" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3472,7 @@
       <c r="O49" s="6" t="n"/>
       <c r="P49" s="6" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3528,7 @@
       <c r="O50" s="8" t="n"/>
       <c r="P50" s="8" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -3586,7 +3584,7 @@
       <c r="O51" s="8" t="n"/>
       <c r="P51" s="8" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -3642,7 +3640,7 @@
       <c r="O52" s="8" t="n"/>
       <c r="P52" s="8" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -3698,7 +3696,7 @@
       <c r="O53" s="8" t="n"/>
       <c r="P53" s="8" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -3754,7 +3752,7 @@
       <c r="O54" s="8" t="n"/>
       <c r="P54" s="8" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -3810,7 +3808,7 @@
       <c r="O55" s="8" t="n"/>
       <c r="P55" s="8" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3864,7 @@
       <c r="O56" s="6" t="n"/>
       <c r="P56" s="6" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -4967,7 +4965,7 @@
       <c r="O76" s="6" t="n"/>
       <c r="P76" s="6" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de contratação de TIC, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
+          <t>formalize e padronize o processo de contratação de TIC, compatível com o porte, a complexidade e os riscos das contratações da organização, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
         </is>
       </c>
     </row>
@@ -5023,7 +5021,7 @@
       <c r="O77" s="6" t="n"/>
       <c r="P77" s="6" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de contratação de TIC, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
+          <t>formalize e padronize o processo de contratação de TIC, compatível com o porte, a complexidade e os riscos das contratações da organização, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
         </is>
       </c>
     </row>
@@ -5079,7 +5077,7 @@
       <c r="O78" s="6" t="n"/>
       <c r="P78" s="6" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de contratação de TIC, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
+          <t>formalize e padronize o processo de contratação de TIC, compatível com o porte, a complexidade e os riscos das contratações da organização, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5133,7 @@
       <c r="O79" s="6" t="n"/>
       <c r="P79" s="6" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de contratação de TIC, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
+          <t>formalize e padronize o processo de contratação de TIC, compatível com o porte, a complexidade e os riscos das contratações da organização, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5189,7 @@
       <c r="O80" s="6" t="n"/>
       <c r="P80" s="6" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de contratação de TIC, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
+          <t>formalize e padronize o processo de contratação de TIC, compatível com o porte, a complexidade e os riscos das contratações da organização, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
         </is>
       </c>
     </row>
@@ -5248,7 +5246,7 @@
       <c r="O81" s="6" t="n"/>
       <c r="P81" s="6" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia e à aprovação técnica da área de TIC, inclusive quando demandadas por outras áreas, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais, a segurança da informação e a arquitetura existente, facultando a adoção de fluxos simplificados ou a dispensa de parecer detalhado para contratações diretas por dispensa em razão do valor (baixo valor) ou de baixa complexidade técnica, mediante critérios objetivos ou catálogos de soluções padronizadas</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, inclusive quando demandadas por outras áreas, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais, a segurança da informação e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
         </is>
       </c>
     </row>
@@ -5818,7 +5816,7 @@
       </c>
       <c r="P92" s="5" t="inlineStr">
         <is>
-          <t>institua formalmente Comitê de TIC ou instância equivalente, atentando-se, minimamente, em definir sua composição, competências, periodicidade de reuniões, forma de registro das deliberações e acompanhamento dos encaminhamentos</t>
+          <t>institua formalmente Comitê de TIC ou instância equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em definir sua composição, competências, periodicidade de reuniões, forma de registro das deliberações e acompanhamento dos encaminhamentos</t>
         </is>
       </c>
     </row>
@@ -5867,7 +5865,7 @@
       </c>
       <c r="P93" s="5" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, atentando-se, minimamente, em realizar reuniões periódicas, registrar atas, deliberações e encaminhamentos e acompanhar as decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em realizar reuniões periódicas, registrar deliberações e acompanhar decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
         </is>
       </c>
     </row>
@@ -5916,7 +5914,7 @@
       </c>
       <c r="P94" s="5" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, atentando-se, minimamente, em realizar reuniões periódicas, registrar atas, deliberações e encaminhamentos e acompanhar as decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em realizar reuniões periódicas, registrar deliberações e acompanhar decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
         </is>
       </c>
     </row>
@@ -5965,7 +5963,7 @@
       </c>
       <c r="P95" s="5" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -6014,7 +6012,7 @@
       </c>
       <c r="P96" s="5" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -6063,7 +6061,7 @@
       </c>
       <c r="P97" s="5" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -6112,7 +6110,7 @@
       </c>
       <c r="P98" s="5" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7363,7 @@
       <c r="O122" s="11" t="n"/>
       <c r="P122" s="10" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -7421,7 +7419,7 @@
       <c r="O123" s="11" t="n"/>
       <c r="P123" s="10" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -7477,7 +7475,7 @@
       <c r="O124" s="11" t="n"/>
       <c r="P124" s="10" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -7533,7 +7531,7 @@
       <c r="O125" s="11" t="n"/>
       <c r="P125" s="10" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -7589,7 +7587,7 @@
       <c r="O126" s="11" t="n"/>
       <c r="P126" s="10" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas para assegurar capacidade interna mínima de coordenação, planejamento, aprovação técnica, fiscalização contratual, tomada de decisão e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente de coordenação, planejamento, aprovação técnica, fiscalização contratual e retenção de conhecimento, especialmente quando a execução das atividades de TIC depender predominantemente de terceiros ou de estrutura externa</t>
         </is>
       </c>
     </row>
@@ -8592,7 +8590,7 @@
       </c>
       <c r="P146" s="5" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de contratação de TIC, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
+          <t>formalize e padronize o processo de contratação de TIC, compatível com o porte, a complexidade e os riscos das contratações da organização, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
         </is>
       </c>
     </row>
@@ -8641,7 +8639,7 @@
       </c>
       <c r="P147" s="5" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de contratação de TIC, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
+          <t>formalize e padronize o processo de contratação de TIC, compatível com o porte, a complexidade e os riscos das contratações da organização, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
         </is>
       </c>
     </row>
@@ -8690,7 +8688,7 @@
       </c>
       <c r="P148" s="5" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de contratação de TIC, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
+          <t>formalize e padronize o processo de contratação de TIC, compatível com o porte, a complexidade e os riscos das contratações da organização, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
         </is>
       </c>
     </row>
@@ -8739,7 +8737,7 @@
       </c>
       <c r="P149" s="5" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de contratação de TIC, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
+          <t>formalize e padronize o processo de contratação de TIC, compatível com o porte, a complexidade e os riscos das contratações da organização, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
         </is>
       </c>
     </row>
@@ -8788,7 +8786,7 @@
       </c>
       <c r="P150" s="5" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de contratação de TIC, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
+          <t>formalize e padronize o processo de contratação de TIC, compatível com o porte, a complexidade e os riscos das contratações da organização, atentando-se, minimamente, em definir fluxo, etapas, papéis, responsabilidades, instâncias de aprovação e modelos de artefatos, manuais, listas de verificação ou orientações internas aplicáveis</t>
         </is>
       </c>
     </row>
@@ -8838,7 +8836,7 @@
       </c>
       <c r="P151" s="5" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia e à aprovação técnica da área de TIC, inclusive quando demandadas por outras áreas, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais, a segurança da informação e a arquitetura existente, facultando a adoção de fluxos simplificados ou a dispensa de parecer detalhado para contratações diretas por dispensa em razão do valor (baixo valor) ou de baixa complexidade técnica, mediante critérios objetivos ou catálogos de soluções padronizadas</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, inclusive quando demandadas por outras áreas, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais, a segurança da informação e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
         </is>
       </c>
     </row>

</xml_diff>